<commit_message>
changes of review 30_12_2024
</commit_message>
<xml_diff>
--- a/temp/contactData (12).xlsx
+++ b/temp/contactData (12).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7050"/>
+    <workbookView windowWidth="20490" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="AddressBook" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>TITLE</t>
   </si>
@@ -65,40 +65,42 @@
     <t>PUBLIC</t>
   </si>
   <si>
-    <t>Mr</t>
-  </si>
-  <si>
-    <t>Anandu</t>
-  </si>
-  <si>
-    <t>kp</t>
-  </si>
-  <si>
-    <t>male</t>
-  </si>
-  <si>
-    <t>anandun1923@gmail.com</t>
-  </si>
-  <si>
-    <t>kollam</t>
-  </si>
-  <si>
-    <t>kd</t>
-  </si>
-  <si>
-    <t>writing,travelling</t>
+    <t>Mr.</t>
+  </si>
+  <si>
+    <t>Jagan</t>
+  </si>
+  <si>
+    <t>Nadh</t>
+  </si>
+  <si>
+    <t>MALE</t>
+  </si>
+  <si>
+    <t>2000-11-21</t>
+  </si>
+  <si>
+    <t>krish123@gmail.com</t>
+  </si>
+  <si>
+    <t>porbandhar</t>
+  </si>
+  <si>
+    <t>gujarat</t>
+  </si>
+  <si>
+    <t>READING,TRAVELLING</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="180" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="22">
     <font>
@@ -723,14 +725,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
@@ -1277,7 +1276,8 @@
     <col min="9" max="9" width="25" customWidth="1"/>
     <col min="10" max="10" width="20" customWidth="1"/>
     <col min="11" max="11" width="50" customWidth="1"/>
-    <col min="12" max="14" width="20" customWidth="1"/>
+    <col min="12" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="60" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -1318,7 +1318,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12">
+    <row r="2" customFormat="1" ht="20" customHeight="1" spans="1:12">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1331,26 +1331,26 @@
       <c r="D2" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="2">
-        <v>36475</v>
-      </c>
-      <c r="F2" s="3" t="s">
+      <c r="E2" t="s">
         <v>16</v>
       </c>
+      <c r="F2" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="G2">
-        <v>9999999999</v>
+        <v>9898989800</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J2">
-        <v>678678</v>
+        <v>689789</v>
       </c>
       <c r="K2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -1358,7 +1358,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" display="anandun1923@gmail.com"/>
+    <hyperlink ref="F2" r:id="rId1" display="krish123@gmail.com"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>